<commit_message>
fix(ppn): native monetary cells and corrected appendix template rows
</commit_message>
<xml_diff>
--- a/resources/ppn_format.xlsx
+++ b/resources/ppn_format.xlsx
@@ -2058,7 +2058,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{B3B167C7-A5FD-4BA3-A2C0-22F546378F49}">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
@@ -2173,13 +2173,13 @@
       <c r="H5" s="25"/>
       <c r="I5" s="3"/>
     </row>
-    <row r="7" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="6" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2300,15 +2300,15 @@
       <c r="J6" s="39"/>
     </row>
     <row r="7" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
+      <c r="A7" s="13"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
     </row>
     <row r="8" spans="1:10" ns3:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -2475,7 +2475,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{831E3701-BDF6-4B80-84B7-72652CFD0248}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -2612,28 +2612,17 @@
       <c r="N6" s="3"/>
     </row>
     <row r="7" spans="1:14" ns3:dyDescent="0.25">
-      <c r="A7" s="1"/>
+      <c r="A7" s="1" t="s">
+        <v>83</v>
+      </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:14" ns3:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
fix: preserve PPN body metadata styles and add bottom-right bugreport contact
</commit_message>
<xml_diff>
--- a/resources/ppn_format.xlsx
+++ b/resources/ppn_format.xlsx
@@ -488,7 +488,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -602,6 +602,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2035,8 +2036,17 @@
       <c r="I14" s="33"/>
       <c r="J14" s="13"/>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <c r="H15"/>
+    <row xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" spans="1:10" s="1" customFormat="1" ns1:dyDescent="0.25">
+      <c r="A15" s="30"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="30"/>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -2299,16 +2309,17 @@
       <c r="I6" s="17"/>
       <c r="J6" s="39"/>
     </row>
-    <row r="7" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A7" s="13"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="40"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
+    <row xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" spans="1:10" ns1:dyDescent="0.25">
+      <c r="A7" s="30"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="30"/>
     </row>
     <row r="8" spans="1:10" ns3:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -2441,16 +2452,17 @@
       <c r="I6" s="45"/>
       <c r="J6" s="39"/>
     </row>
-    <row r="7" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
+    <row xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" spans="1:10" ns1:dyDescent="0.25">
+      <c r="A7" s="30"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="30"/>
     </row>
     <row r="8" spans="1:10" ns3:dyDescent="0.25">
       <c r="A8" s="1" t="s">

</xml_diff>

<commit_message>
fix(ppn): numeric amounts, corrected body rows and bugreport footer (#29)
* test(ppn): specify numeric amounts and clean body-row formatting (RED)

* fix(ppn): native monetary cells and corrected appendix template rows

* test: cover A2 and B3 review findings and isolate Tk scaling

* fix: preserve PPN body metadata styles and add bottom-right bugreport contact

* test: record approved literal bugreport contact in copy contract

---------

Co-authored-by: Punto Ami Priyono <189459396+cepeter@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resources/ppn_format.xlsx
+++ b/resources/ppn_format.xlsx
@@ -488,7 +488,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -602,6 +602,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -2035,8 +2036,17 @@
       <c r="I14" s="33"/>
       <c r="J14" s="13"/>
     </row>
-    <row r="15" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <c r="H15"/>
+    <row xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" spans="1:10" s="1" customFormat="1" ns1:dyDescent="0.25">
+      <c r="A15" s="30"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="47"/>
+      <c r="G15" s="47"/>
+      <c r="H15" s="47"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="30"/>
     </row>
     <row r="16" spans="1:10" s="1" customFormat="1" ns3:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -2058,7 +2068,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{B3B167C7-A5FD-4BA3-A2C0-22F546378F49}">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
@@ -2173,13 +2183,13 @@
       <c r="H5" s="25"/>
       <c r="I5" s="3"/>
     </row>
-    <row r="7" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="6" spans="1:15" s="1" customFormat="1" ns3:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2299,16 +2309,17 @@
       <c r="I6" s="17"/>
       <c r="J6" s="39"/>
     </row>
-    <row r="7" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
+    <row xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" spans="1:10" ns1:dyDescent="0.25">
+      <c r="A7" s="30"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="30"/>
     </row>
     <row r="8" spans="1:10" ns3:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -2441,16 +2452,17 @@
       <c r="I6" s="45"/>
       <c r="J6" s="39"/>
     </row>
-    <row r="7" spans="1:10" ns3:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
+    <row xmlns:ns1="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" spans="1:10" ns1:dyDescent="0.25">
+      <c r="A7" s="30"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="30"/>
     </row>
     <row r="8" spans="1:10" ns3:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -2475,7 +2487,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{831E3701-BDF6-4B80-84B7-72652CFD0248}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15" ns3:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -2612,28 +2624,17 @@
       <c r="N6" s="3"/>
     </row>
     <row r="7" spans="1:14" ns3:dyDescent="0.25">
-      <c r="A7" s="1"/>
+      <c r="A7" s="1" t="s">
+        <v>83</v>
+      </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:14" ns3:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>